<commit_message>
Correlaciones, laminas regionales y nacionales, payloads y manifiestos
Correlaciones recalculadas sobre 333 comunas (antes 331). Educacion con su
media nacional de 2022 y la serie historica completa. Ocupacion con el tramo de
60 y mas en una sola serie.
</commit_message>
<xml_diff>
--- a/output/graficos_educacion_tasas/comunal_e_mat_a_2018_antofagasta.xlsx
+++ b/output/graficos_educacion_tasas/comunal_e_mat_a_2018_antofagasta.xlsx
@@ -27,30 +27,30 @@
     <t xml:space="preserve">Antofagasta</t>
   </si>
   <si>
+    <t xml:space="preserve">Mejillones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sierra Gorda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taltal</t>
+  </si>
+  <si>
     <t xml:space="preserve">Calama</t>
   </si>
   <si>
+    <t xml:space="preserve">Ollagüe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Pedro de Atacama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tocopilla</t>
+  </si>
+  <si>
     <t xml:space="preserve">María Elena</t>
   </si>
   <si>
-    <t xml:space="preserve">Mejillones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ollagüe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Pedro de Atacama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sierra Gorda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taltal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tocopilla</t>
-  </si>
-  <si>
     <t xml:space="preserve">Campo</t>
   </si>
   <si>
@@ -60,7 +60,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-09 20:21</t>
+    <t xml:space="preserve">2026-09-18 10:12</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -480,7 +480,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>67.56</v>
+        <v>64.65</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>67.2</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="5">
@@ -496,7 +496,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>64.65</v>
+        <v>73.22</v>
       </c>
     </row>
     <row r="6">
@@ -504,7 +504,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>72.86</v>
+        <v>67.56</v>
       </c>
     </row>
     <row r="7">
@@ -512,7 +512,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>66.85</v>
+        <v>72.86</v>
       </c>
     </row>
     <row r="8">
@@ -520,7 +520,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>66.67</v>
+        <v>66.85</v>
       </c>
     </row>
     <row r="9">
@@ -528,7 +528,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>73.22</v>
+        <v>69.47</v>
       </c>
     </row>
     <row r="10">
@@ -536,7 +536,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>69.47</v>
+        <v>67.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>